<commit_message>
chore: run 2026-09-14 20:42 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_14_09_2026.xlsx
+++ b/logs/Consolidado_14_09_2026.xlsx
@@ -657,7 +657,7 @@
         <v>154</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -676,10 +676,10 @@
         <v>69</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
@@ -695,7 +695,7 @@
         <v>79</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -714,7 +714,7 @@
         <v>68</v>
       </c>
       <c r="C5" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -733,10 +733,10 @@
         <v>48</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
@@ -752,10 +752,10 @@
         <v>102</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>6</v>
@@ -4995,37 +4995,37 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="7" t="inlineStr">
+      <c r="A113" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="B113" s="7" t="inlineStr">
+      <c r="B113" s="5" t="inlineStr">
         <is>
           <t>Cleanance Cleansing Gel</t>
         </is>
       </c>
-      <c r="C113" s="7" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="D113" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E113" s="7" t="inlineStr">
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
         <is>
           <t>6552595</t>
         </is>
       </c>
-      <c r="F113" s="7" t="inlineStr">
+      <c r="F113" s="5" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="G113" s="7" t="inlineStr">
+      <c r="G113" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-cleansing-gel-443317.html</t>
         </is>
@@ -20057,7 +20057,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>8726970</t>
+        </is>
+      </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
           <t>25%</t>
@@ -20189,42 +20193,42 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Cleanance Cleansing Gel</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-cleansing-gel-443317.html</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>6552595</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
@@ -21184,7 +21188,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr"/>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>3599509</t>
+        </is>
+      </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
           <t>25%</t>
@@ -21472,40 +21480,40 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C58" s="7" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Dermabsolu Eco-Refill Redensifying Day Cream
 Recarga Creme anti idade Rugas e Firmeza
 50 ml</t>
         </is>
       </c>
-      <c r="D58" s="7" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/dermabsolu-eco-refill-redensifying-day-cream-8152747.html</t>
         </is>
       </c>
-      <c r="E58" s="7" t="inlineStr"/>
-      <c r="F58" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>8152747</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -21540,7 +21548,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>6739622</t>
+        </is>
+      </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
           <t>25%</t>
@@ -24713,7 +24725,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G138" s="3" t="inlineStr"/>
+      <c r="G138" s="3" t="inlineStr">
+        <is>
+          <t>7378122</t>
+        </is>
+      </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
           <t>25%</t>
@@ -27020,40 +27036,40 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Kelual DS Gel Nettoyant Anti-squames
 Gel Limpeza Dermatite Seborreica
 200 ml</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/kelual-ds-gel-nettoyant-anti-squames-8226845.html</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr"/>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>8226845</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -27994,40 +28010,40 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Kertyol PSO Daily Balm
 Bálsamo Corpo Hidratante Pele com Psoríase
 200 ml</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/kertyol-pso-daily-balm-8487355.html</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr"/>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>8487355</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -28114,40 +28130,40 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Kit Anaphase Anti-Hair Loss and Growth
 Champô Queda de Cabelo Reativa com Oferta
 1 un</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/kit-anaphase-anti-hair-loss-and-growth-8640386.html</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>8640386</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -29994,40 +30010,40 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Cupuaçu Repairing Restorative CICA-Serum
 Sérum Cupuaçu Repara Cabelo Muito Seco
 100 ml</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cupuacu-repairing-restorative-cica-serum-8557935.html</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr"/>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>8557935</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -33499,40 +33515,40 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Curbicia Scalp Prone to Oiliness Shampoo
 Champô Equilibrante Couro Cabeludo Oleoso
 150 ml</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/curbicia-scalp-prone-to-oiliness-shampoo-5520011.html</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>5520011</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -34673,40 +34689,40 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>Style Sculpting Mousse Volume &amp; Sculpt
 Espuma Cabelo Modeladora Volumizadora da Raiz
 200 ml</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/style-sculpting-mousse-volume-and-sculpt-7447302.html</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr"/>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
         <is>
           <t>7447302</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -34793,40 +34809,40 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Sublime Curl Activating Detangling Conditioner
 Condicionador Suave e Redefinidor de Caracóis
 150 ml</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-curl-activating-detangling-conditioner-5972162.html</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr"/>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>5972162</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -35439,40 +35455,40 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B65" s="7" t="inlineStr">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C65" s="7" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>Triphasic Anti-Hair Loss Shampoo
 Champô Queda de Cabelo com Óleos Essenciais
 50 ml</t>
         </is>
       </c>
-      <c r="D65" s="7" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-anti-hair-loss-shampoo-7630904.html</t>
         </is>
       </c>
-      <c r="E65" s="7" t="inlineStr"/>
-      <c r="F65" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G65" s="7" t="inlineStr">
+      <c r="E65" s="3" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>7630904</t>
         </is>
       </c>
-      <c r="H65" s="7" t="inlineStr">
+      <c r="H65" s="3" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
@@ -36068,40 +36084,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Biology AC Purifying Cleansing Foaming Gel
 Gel Espuma de Limpeza Purificante para Acne
 200 ml</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/biology-ac-purifying-cleansing-foaming-gel-7756106.html</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>7756106</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -39140,40 +39156,40 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Elgydium
 Escova de Dentes 20 100 Soft
 1 un</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/escova-de-dentes-20-100-soft-4031126.html</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>4031126</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-09-14 21:19 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_14_09_2026.xlsx
+++ b/logs/Consolidado_14_09_2026.xlsx
@@ -695,7 +695,7 @@
         <v>79</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -29571,39 +29571,39 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Champô Antiqueda Quinina Edelvaisse + Oferta
 200 ml + 100 ml</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/champo-antiqueda-quinina-edelvaisse-oferta-7834045.html</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>7834045</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>

</xml_diff>